<commit_message>
feat: designate v4 as master workbook template
</commit_message>
<xml_diff>
--- a/fixtures/IT_Exec_Reporting_Ingestion_Template_v4_dummy_data.xlsx
+++ b/fixtures/IT_Exec_Reporting_Ingestion_Template_v4_dummy_data.xlsx
@@ -874,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -884,14 +884,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IT Exec Reporting — Ingestion Template</t>
+          <t>IT Reporting — Master Ingestion Template</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Use this workbook as the future ingestion layer for the exec-level IT report. Each INPUT_ sheet represents one reporting domain. Keep one row per metric, item, ticket, project or roadmap entry as appropriate.</t>
+          <t>This is the master workbook contract for the TeacherActive IT Reporting pack. Keep worksheet names, row 3 headers and Excel table names exact so the app can ingest the file reliably.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12-week rolling Gantt is derived from INPUT_Portfolio_Gantt_Workstreams and INPUT_Portfolio_Gantt_Milestones.</t>
+          <t>12-week rolling Gantt is derived from INPUT_Gantt_Workstreams and INPUT_Gantt_Milestones.</t>
         </is>
       </c>
     </row>
@@ -1129,12 +1129,108 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Master template status</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>This workbook is the current master ingestion template for the IT Reporting pack. Use it for all new monthly packs unless a newer template version is formally issued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Workbook authority</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>The app expects the exact worksheet names, row 3 headers and Excel table names defined in this workbook. Do not rename sheets, move the header row, or remove tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Input tab rule</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Populate INPUT_ tabs and Periods only. Reporting_Framework, Metric_Catalogue and Validation_Lists are reference tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Exec Summary handling</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Exec Summary is authored in the app, not in Excel. The workbook remains the source of truth for structured reporting data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Map handling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Office map plotting uses app-owned coordinates. Office_Locations Map X and Map Y remain reference fields and are not the live plotting source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Chart settings handling</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Chart overlays are controlled in INPUT_Chart_Settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Required input sheets</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Periods, INPUT_Office_Network_Avail, INPUT_Service_Availability, INPUT_Support_Operations, INPUT_Top_Oldest_Tickets, INPUT_Security_Patching, INPUT_Assets_Lifecycle, INPUT_Change_Release, INPUT_Dev_Delivery, INPUT_Project_Portfolio, INPUT_Rolling_Roadmap, INPUT_Gantt_Workstreams, INPUT_Gantt_Milestones, INPUT_Budget_Commercials, INPUT_Top_Risks, INPUT_Narrative_Notes, INPUT_Chart_Settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Required table names</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TOfficeLocations, TOfficeNetworkAvailability, TServiceAvailability, TSupportOperations, TTopOldestTickets, TSecurityPatching, TAssetsLifecycle, TChangeRelease, TDevDelivery, TProjectPortfolio, TRollingRoadmap, TPortfolioGanttWorkstreams, TPortfolioGanttMilestones, TBudgetCommercials, TTopRisks, TNarrativeNotes, TChartSettings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Periods sheet rule</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Periods must contain Report Cut-Off Date on row 3 and exactly one current period marked Yes.</t>
         </is>
       </c>
     </row>

</xml_diff>